<commit_message>
various corrections for WGEEL 2026
</commit_message>
<xml_diff>
--- a/R/advice/table3.xlsx
+++ b/R/advice/table3.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuille1" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Feuille1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="21">
   <si>
     <t xml:space="preserve">Year</t>
   </si>
@@ -97,6 +97,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -118,11 +119,13 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Calibri"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -191,23 +194,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -283,13 +286,119 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="FFFFFF"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18A303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369A3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A33E03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8E03A3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="C99C00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="C9211E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000EE"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551A8B"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E30"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -735,10 +844,19 @@
       <c r="A29" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="B29" s="3"/>
-      <c r="C29" s="4"/>
+      <c r="B29" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="D29" s="5"/>
       <c r="E29" s="5"/>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="n">
+        <v>2027</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>